<commit_message>
docs: add real defect retest evidence and edge smoke coverage
</commit_message>
<xml_diff>
--- a/Report Test subject/Powered by GPT/TestCases/UI/OSMS-UI-Test-Cases.xlsx
+++ b/Report Test subject/Powered by GPT/TestCases/UI/OSMS-UI-Test-Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\Online-Sales-Management-System\Report Test subject\Powered by GPT\TestCases\UI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{83BAF67A-3631-403B-91B8-B20F51886819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3461925E-C669-4F72-AD20-6C3944B89B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{734EF4B4-F574-4C8E-BC30-443F83F1EC28}"/>
   </bookViews>
@@ -116,15 +116,9 @@
     <t>User is redirected to the admin area dashboard; authenticated session is established; no validation error is shown.</t>
   </si>
   <si>
-    <t>Valid admin login reached the admin dashboard successfully in the focused Selenium rerun.</t>
-  </si>
-  <si>
     <t>Pass</t>
   </si>
   <si>
-    <t>TestResults/Evidence/UI/automation/20260406_053930_TC-UI-AUTH-001-success.png ; TestResults/RunnerOutput/UI/auth-permission-rerun.trx ; Videos/OSMS-Automation-Demo.mp4</t>
-  </si>
-  <si>
     <t>TC-UI-AUTH-002</t>
   </si>
   <si>
@@ -320,15 +314,9 @@
     <t>Invoice is created successfully; details page is shown; invoice status is Unpaid; stock is reduced by the sold quantity.</t>
   </si>
   <si>
-    <t>Submitting a valid walk-in invoice returned to the Create page with the toast message Failed to create invoice. Please check data and try again. Server log confirms InvalidOperationException caused by a user-initiated transaction with MySqlRetryingExecutionStrategy in InvoicesController.Create line 145.</t>
-  </si>
-  <si>
     <t>Fail</t>
   </si>
   <si>
-    <t>TestResults/Evidence/UI/automation/20260406_053902_TC-UI-INV-001-failure.png ; TestResults/RunnerOutput/UI/invoice-rerun.trx ; TestResults/Defects/OSMS-Defect-Log.xlsx ; https://github.com/Alucard30Dec/Online-Sales-Management-System/issues/1</t>
-  </si>
-  <si>
     <t>TC-UI-INV-002</t>
   </si>
   <si>
@@ -431,12 +419,6 @@
     <t>Invoice status becomes Cancelled; stock increases by the cancelled quantity; a stock movement entry is recorded.</t>
   </si>
   <si>
-    <t>Cancelling the invoice failed on the details page with the toast Failed to cancel invoice. Please try again., so the invoice was not cancelled and stock was not returned.</t>
-  </si>
-  <si>
-    <t>TestResults/Evidence/UI/automation/20260411_075908_TC-UI-INV-005-failure.png ; TestResults/RunnerOutput/UI/reporting-public-invoice-coverage.trx</t>
-  </si>
-  <si>
     <t>TC-UI-REP-001</t>
   </si>
   <si>
@@ -656,12 +638,6 @@
     <t>Purchase is not created; supplier validation error is shown.</t>
   </si>
   <si>
-    <t>Purchase was not created, but the create page only rendered a blank red validation banner instead of a readable supplier-required error message.</t>
-  </si>
-  <si>
-    <t>TestResults/Evidence/UI/automation/20260410_113408_TC-UI-PUR-002-failure.png ; TestResults/RunnerOutput/UI/purchase-product-import-coverage-rerun.trx</t>
-  </si>
-  <si>
     <t>TC-UI-PUR-003</t>
   </si>
   <si>
@@ -1019,12 +995,6 @@
     <t>Import completes successfully; success toast is shown; imported or updated products appear in product list.</t>
   </si>
   <si>
-    <t>After a valid preview, import confirm returned to the import page with the toast Import thất bại. Vui lòng thử lại., and the expected imported product did not appear in the product list.</t>
-  </si>
-  <si>
-    <t>TestResults/Evidence/UI/automation/20260410_113328_TC-UI-IMP-003-failure.png ; TestResults/RunnerOutput/UI/purchase-product-import-coverage-rerun.trx</t>
-  </si>
-  <si>
     <t>TC-UI-IMP-004</t>
   </si>
   <si>
@@ -1293,6 +1263,36 @@
   </si>
   <si>
     <t>TestResults/Evidence/UI/automation/20260410_102600_TC-UI-PUB-003-details.png ; TestResults/RunnerOutput/UI/tc-ui-pub-003-rerun.trx</t>
+  </si>
+  <si>
+    <t>TestResults/Evidence/UI/automation/20260406_053930_TC-UI-AUTH-001-success.png ; TestResults/Evidence/UI/automation/20260411_143741_TC-UI-AUTH-001-success.png ; TestResults/RunnerOutput/UI/auth-permission-rerun.trx ; TestResults/RunnerOutput/UI/edge-auth-smoke.trx ; Videos/OSMS-Automation-Demo.mp4</t>
+  </si>
+  <si>
+    <t>Valid admin login reached the admin dashboard successfully in both the focused Chrome rerun and a secondary Edge smoke rerun on 2026-04-11.</t>
+  </si>
+  <si>
+    <t>TestResults/Evidence/UI/automation/20260406_053902_TC-UI-INV-001-failure.png ; TestResults/Evidence/UI/automation/20260411_143458_TC-UI-INV-001-failure.png ; TestResults/RunnerOutput/UI/invoice-rerun.trx ; TestResults/RunnerOutput/UI/postfix-retest-inv-001.trx ; TestResults/Defects/OSMS-Defect-Log.xlsx ; https://github.com/Alucard30Dec/Online-Sales-Management-System/issues/1</t>
+  </si>
+  <si>
+    <t>Submitting a valid walk-in invoice returned to the Create page with the toast message Failed to create invoice. Please check data and try again. Server log confirms InvalidOperationException caused by a user-initiated transaction with MySqlRetryingExecutionStrategy in InvoicesController.Create line 145. A focused rerun on 2026-04-11 still failed before reaching the details page, so the defect remains reproducible.</t>
+  </si>
+  <si>
+    <t>TestResults/Evidence/UI/automation/20260411_075908_TC-UI-INV-005-failure.png ; TestResults/Evidence/UI/automation/20260411_143548_TC-UI-INV-005-failure.png ; TestResults/RunnerOutput/UI/reporting-public-invoice-coverage.trx ; TestResults/RunnerOutput/UI/postfix-retest-inv-005.trx ; https://github.com/Alucard30Dec/Online-Sales-Management-System/issues/4</t>
+  </si>
+  <si>
+    <t>Cancelling the invoice failed on the details page with the toast Failed to cancel invoice. Please try again., so the invoice was not cancelled and stock was not returned. A focused rerun on 2026-04-11 reproduced the same cancellation failure.</t>
+  </si>
+  <si>
+    <t>TestResults/Evidence/UI/automation/20260410_113408_TC-UI-PUR-002-failure.png ; TestResults/Evidence/UI/automation/20260411_143535_TC-UI-PUR-002-failure.png ; TestResults/RunnerOutput/UI/purchase-product-import-coverage-rerun.trx ; TestResults/RunnerOutput/UI/postfix-retest-pur-002.trx ; https://github.com/Alucard30Dec/Online-Sales-Management-System/issues/2</t>
+  </si>
+  <si>
+    <t>Purchase was not created, but the create page only rendered a blank red validation banner instead of a readable supplier-required error message. A focused rerun on 2026-04-11 reproduced the same unreadable validation banner.</t>
+  </si>
+  <si>
+    <t>TestResults/Evidence/UI/automation/20260410_113328_TC-UI-IMP-003-failure.png ; TestResults/Evidence/UI/automation/20260411_143540_TC-UI-IMP-003-failure.png ; TestResults/RunnerOutput/UI/purchase-product-import-coverage-rerun.trx ; TestResults/RunnerOutput/UI/postfix-retest-imp-003.trx ; https://github.com/Alucard30Dec/Online-Sales-Management-System/issues/3</t>
+  </si>
+  <si>
+    <t>After a valid preview, import confirm returned to the import page with the toast Import th?t b?i. Vui l?ng th? l?i., and the expected imported product did not appear in the product list. A focused rerun on 2026-04-11 reproduced the same failure.</t>
   </si>
 </sst>
 </file>
@@ -1776,24 +1776,24 @@
         <v>24</v>
       </c>
       <c r="L2" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="N2" s="2" t="s">
-        <v>27</v>
+        <v>408</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="375" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>30</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>17</v>
@@ -1808,39 +1808,39 @@
         <v>20</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="M3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="L3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N3" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>18</v>
@@ -1852,39 +1852,39 @@
         <v>20</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="M4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:14" ht="225" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="M4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N4" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>18</v>
@@ -1896,39 +1896,39 @@
         <v>20</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="K5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="M5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N5" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="K5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="L5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:14" ht="281.25" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N5" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="337.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>58</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>18</v>
@@ -1937,42 +1937,42 @@
         <v>19</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="K6" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="L6" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="M6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N6" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="L6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="M6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N6" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" ht="375" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>68</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>18</v>
@@ -1981,42 +1981,42 @@
         <v>19</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H7" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="L7" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="M7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N7" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="L7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="M7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>78</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>18</v>
@@ -2025,42 +2025,42 @@
         <v>19</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H8" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="L8" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="M8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>86</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>18</v>
@@ -2072,39 +2072,39 @@
         <v>20</v>
       </c>
       <c r="H9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="L9" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="M9" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="K9" s="2" t="s">
+      <c r="N9" s="2" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="225" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="M9" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="N9" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>98</v>
-      </c>
       <c r="D10" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>18</v>
@@ -2116,39 +2116,39 @@
         <v>20</v>
       </c>
       <c r="H10" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="M10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N10" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="J10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:14" ht="281.25" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="M10" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N10" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="D11" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>18</v>
@@ -2160,39 +2160,39 @@
         <v>20</v>
       </c>
       <c r="H11" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="L11" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="M11" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="N11" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="J11" s="2" t="s">
+    </row>
+    <row r="12" spans="1:14" ht="318.75" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="K11" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="M11" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="D12" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>18</v>
@@ -2204,39 +2204,39 @@
         <v>20</v>
       </c>
       <c r="H12" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="L12" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="M12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>18</v>
@@ -2248,39 +2248,39 @@
         <v>20</v>
       </c>
       <c r="H13" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="300" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="J13" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="375" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>18</v>
@@ -2289,42 +2289,42 @@
         <v>19</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H14" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="300" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="B15" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N14" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="D15" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>18</v>
@@ -2333,1183 +2333,1183 @@
         <v>19</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H15" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="K15" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="L15" s="2" t="s">
+      <c r="E16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="M15" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N15" s="2" t="s">
+      <c r="G16" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" ht="318.75" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
+      <c r="I16" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="K16" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="L16" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="M16" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N16" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H16" s="2" t="s">
+    </row>
+    <row r="17" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="B17" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="J16" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="K16" s="2" t="s">
+      <c r="D17" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="L16" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="M16" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N16" s="2" t="s">
+      <c r="K17" s="2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" ht="356.25" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
+      <c r="L17" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="M17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N17" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C17" s="2" t="s">
+    </row>
+    <row r="18" spans="1:14" ht="225" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="I17" s="2" t="s">
+      <c r="B18" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="J17" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="K17" s="2" t="s">
+      <c r="J18" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="L17" s="2" t="s">
+      <c r="K18" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="M17" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N17" s="2" t="s">
+      <c r="L18" s="2" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" ht="356.25" x14ac:dyDescent="0.3">
-      <c r="A18" s="2" t="s">
+      <c r="M18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N18" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="C18" s="2" t="s">
+    </row>
+    <row r="19" spans="1:14" ht="318.75" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="I18" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="J18" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="K18" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="L18" s="2" t="s">
+      <c r="E19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="M18" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N18" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" ht="337.5" x14ac:dyDescent="0.3">
-      <c r="A19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="K19" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="L19" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G19" s="2" t="s">
+      <c r="M19" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N19" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="H19" s="2" t="s">
+    </row>
+    <row r="20" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="J19" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="K19" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="L19" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N19" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>191</v>
-      </c>
       <c r="E20" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H20" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="I20" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="J20" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="L20" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N20" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="375" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>200</v>
-      </c>
       <c r="D21" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>205</v>
+        <v>415</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="262.5" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H22" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="I22" s="2" t="s">
-        <v>209</v>
-      </c>
       <c r="J22" s="2" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="375" x14ac:dyDescent="0.3">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="318.75" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H23" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="L23" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="281.25" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="I23" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="L23" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>225</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="262.5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H25" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="L25" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="M25" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="225" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H26" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="I26" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="J25" s="2" t="s">
+      <c r="J26" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="K25" s="2" t="s">
+      <c r="K26" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="L25" s="2" t="s">
+      <c r="L26" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="M25" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N25" s="2" t="s">
+      <c r="M26" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H26" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="E27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="J26" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>245</v>
-      </c>
-      <c r="L26" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>251</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H27" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="M27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="I27" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" ht="375" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>259</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>260</v>
-      </c>
       <c r="D28" s="2" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H28" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="L28" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="M28" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" ht="206.25" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="I28" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>263</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>265</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" ht="337.5" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>267</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>269</v>
-      </c>
       <c r="D29" s="2" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G29" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" ht="356.25" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="225" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H30" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="I30" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="I30" s="2" t="s">
+      <c r="J30" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="M30" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="J30" s="2" t="s">
+      <c r="I31" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="K30" s="2" t="s">
+      <c r="J31" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="L30" s="2" t="s">
+      <c r="K31" s="2" t="s">
         <v>281</v>
       </c>
-      <c r="M30" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N30" s="2" t="s">
+      <c r="L31" s="2" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A31" s="2" t="s">
+      <c r="M31" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N31" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="B31" s="2" t="s">
+    </row>
+    <row r="32" spans="1:14" ht="262.5" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="B32" s="2" t="s">
         <v>285</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H31" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="I31" s="2" t="s">
+      <c r="D32" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>287</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="I32" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="K31" s="2" t="s">
+      <c r="J32" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="L31" s="2" t="s">
+      <c r="K32" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="M31" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N31" s="2" t="s">
+      <c r="L32" s="2" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
+      <c r="M32" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N32" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="B32" s="2" t="s">
+    </row>
+    <row r="33" spans="1:14" ht="206.25" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H32" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="D33" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="J32" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N32" s="2" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" ht="375" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>304</v>
-      </c>
       <c r="E33" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G33" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="262.5" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
     </row>
     <row r="35" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>326</v>
+        <v>417</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="281.25" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H36" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H37" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="I37" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="J37" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="K36" s="2" t="s">
+      <c r="K37" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="L36" s="2" t="s">
+      <c r="L37" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="M36" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N36" s="2" t="s">
+      <c r="M37" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N37" s="2" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="356.25" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
+    <row r="38" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="B37" s="2" t="s">
+      <c r="B38" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="C38" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="D38" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H38" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H37" s="2" t="s">
+      <c r="I38" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="J38" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="J37" s="2" t="s">
+      <c r="K38" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="L38" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="L37" s="2" t="s">
+      <c r="M38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N38" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="M37" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N37" s="2" t="s">
+    </row>
+    <row r="39" spans="1:14" ht="300" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
+      <c r="B39" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="D39" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H39" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="I39" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H38" s="2" t="s">
+      <c r="J39" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="I38" s="2" t="s">
+      <c r="K39" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="J38" s="2" t="s">
+      <c r="L39" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="K38" s="2" t="s">
+      <c r="M39" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N39" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="L38" s="2" t="s">
+    </row>
+    <row r="40" spans="1:14" ht="243.75" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="M38" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N38" s="2" t="s">
+      <c r="B40" s="2" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A39" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>347</v>
-      </c>
-      <c r="C39" s="2" t="s">
+      <c r="D40" s="2" t="s">
         <v>356</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H39" s="2" t="s">
+      <c r="E40" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="F40" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H40" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="J39" s="2" t="s">
+      <c r="I40" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="J40" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="L39" s="2" t="s">
+      <c r="K40" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="M39" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N39" s="2" t="s">
+      <c r="L40" s="2" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
+      <c r="M40" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N40" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="B40" s="2" t="s">
+    </row>
+    <row r="41" spans="1:14" ht="262.5" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="B41" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" ht="375" x14ac:dyDescent="0.3">
-      <c r="A41" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>376</v>
-      </c>
       <c r="D41" s="2" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>367</v>
+        <v>357</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H41" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="J41" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="I41" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>378</v>
-      </c>
       <c r="K41" s="2" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="42" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" ht="281.25" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>17</v>
@@ -3521,42 +3521,42 @@
         <v>19</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="43" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" ht="281.25" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>392</v>
+        <v>382</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>18</v>
@@ -3565,116 +3565,116 @@
         <v>19</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>394</v>
+        <v>384</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>395</v>
+        <v>385</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>396</v>
+        <v>386</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>398</v>
+        <v>388</v>
       </c>
       <c r="M43" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="44" spans="1:14" ht="409.5" x14ac:dyDescent="0.3">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>402</v>
+        <v>392</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>18</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>20</v>
       </c>
       <c r="H44" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" ht="337.5" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="I45" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="I44" s="2" t="s">
+      <c r="J45" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="J44" s="2" t="s">
+      <c r="K45" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="K44" s="2" t="s">
+      <c r="L45" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="L44" s="2" t="s">
+      <c r="M45" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N45" s="2" t="s">
         <v>407</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="N44" s="2" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="45" spans="1:14" ht="393.75" x14ac:dyDescent="0.3">
-      <c r="A45" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>410</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>411</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="I45" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="J45" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="K45" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="L45" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="M45" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="N45" s="2" t="s">
-        <v>417</v>
       </c>
     </row>
   </sheetData>

</xml_diff>